<commit_message>
Preserve roster start dates and support all pilot holdings in the member editor
</commit_message>
<xml_diff>
--- a/docs/members.example.xlsx
+++ b/docs/members.example.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Members'!$A$1:$N$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Members'!$A$1:$O$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,8 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="hh:mm"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -66,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -75,6 +76,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -443,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -460,6 +462,7 @@
     <col width="24" customWidth="1" min="12" max="12"/>
     <col width="30" customWidth="1" min="13" max="13"/>
     <col width="55" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -533,6 +536,11 @@
           <t>feedback</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>delivery_start_date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -599,9 +607,10 @@
           <t>Example only. Replace this row with reviewed member details.</t>
         </is>
       </c>
+      <c r="O2" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N2"/>
+  <autoFilter ref="A1:O2"/>
   <dataValidations count="2">
     <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Choose participation" error="Use true/yes only after reviewing email participation." type="list" errorStyle="stop">
       <formula1>"true,false,yes,no"</formula1>
@@ -621,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -629,168 +638,180 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Topic</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Instructions</t>
         </is>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Pilot cadence</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>The pilot sends one email per member per week. Survey frequency preferences do not change the scheduler.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Paper slips</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Transcribe the original answers into the optional preference and feedback columns. Keep operational choices separate.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Example row</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Replace the example before enrollment. It is disabled and uses an example.com address.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Stable ID</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Use a unique stable id for each person. Preserve it when editing names or email addresses.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Groups and holdings</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Use semicolons between groups or ticker symbols. Personal tickers replace group defaults; blank inherits defaults.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Participation</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>enabled controls weekly email. A contact-interest checkbox alone does not automatically enable sending.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Time zone</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>The paper form uses Toronto time. Use America/Toronto unless the member confirms a different zone.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Exact time</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>send_time needs HH:MM. Before 9 AM or After 5 PM belongs in preferred_time until an exact time is confirmed.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Weekday</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>send_weekday is one confirmed day: Monday=0, Tuesday=1, Wednesday=2, Thursday=3, Friday=4, Saturday=5, Sunday=6.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Delivery start date</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Optional delivery_start_date uses YYYY-MM-DD. Only weekly occurrences on or after this date are eligible. A blank date allows the current weekly occurrence, including catch-up after its scheduled time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="44" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Optional survey data</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>preferred_frequency, preferred_weekdays, preferred_time, content_preferences and feedback are retained privately, not interpreted as delivery instructions.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="44" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="13" ht="44" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Privacy</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Keep the completed workbook private. Do not commit real names or addresses to the repository.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="44" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="14" ht="44" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Import</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>python scripts/subscriptions.py config/subscriptions.local.json --import-excel config/members.local.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="44" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15" ht="44" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Activation</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Importing does not send email. Review private previews and enable the workflow separately.</t>
         </is>

</xml_diff>